<commit_message>
aggiornamento di fine sprint
</commit_message>
<xml_diff>
--- a/7_Allegati/Sprint_Planning.xlsx
+++ b/7_Allegati/Sprint_Planning.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Scuola\Anno_3\Modulo_306\System-Breach-Five-Nights\7_Allegati\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E83CED4-3463-4DB5-8E62-3CA571A7D9B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7E63F8-E11E-4AC4-905F-94D8C0EE6BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{BE00B4A7-9DBD-4145-8685-CE8529F262A7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="24">
   <si>
     <t>Sprint 1</t>
   </si>
@@ -77,9 +77,6 @@
     <t>implementare attacco THE SINGULARITY</t>
   </si>
   <si>
-    <t>implementare salvataggio partita/impostazioni</t>
-  </si>
-  <si>
     <t>Sprint 4</t>
   </si>
   <si>
@@ -105,6 +102,12 @@
   </si>
   <si>
     <t>implementare meccanismo di difesa firewall</t>
+  </si>
+  <si>
+    <t>10h</t>
+  </si>
+  <si>
+    <t>implementare salvataggio impostazioni e partita</t>
   </si>
 </sst>
 </file>
@@ -127,12 +130,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -162,15 +171,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="17">
     <dxf>
       <font>
         <color rgb="FF92D050"/>
@@ -192,6 +202,46 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF92D050"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92D050"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92D050"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF92D050"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FF00B050"/>
@@ -209,6 +259,16 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF92D050"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FF00B050"/>
@@ -226,46 +286,46 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FF92D050"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -609,7 +669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0104325A-DF2A-4DED-A323-01FD57F9E384}">
-  <dimension ref="A1:BN21"/>
+  <dimension ref="A1:BN24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="47.77734375" bestFit="1" customWidth="1"/>
@@ -708,7 +768,7 @@
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
-        <v>11h</v>
+        <v>9h</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>3</v>
@@ -735,12 +795,6 @@
         <v>3</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="S4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="T4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -750,7 +804,7 @@
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
-        <v>11h</v>
+        <v>9h</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>3</v>
@@ -777,12 +831,6 @@
         <v>3</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="S5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="T5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -863,422 +911,383 @@
     </row>
     <row r="8" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" t="str">
-        <f t="shared" ref="B8:B21" si="1">_xlfn.CONCAT(COUNTIF($C8:$XFD8,"x"),"h")</f>
-        <v>16h</v>
-      </c>
-      <c r="U8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="V8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="W8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="X8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AB8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AG8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AI8" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="T8" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:50" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" ref="B9:B17" si="1">_xlfn.CONCAT(COUNTIF($C9:$XFD9,"x"),"h")</f>
+        <v>14h</v>
+      </c>
+      <c r="U9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="W9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="X9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH9" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="1"/>
+        <v>14h</v>
+      </c>
+      <c r="U10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="W10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="X10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Y10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG10" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH10" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>21</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B11" t="str">
+        <f t="shared" si="1"/>
+        <v>2h</v>
+      </c>
+      <c r="AG11" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH11" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="1"/>
+        <v>2h</v>
+      </c>
+      <c r="AG12" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH12" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="1"/>
+        <v>7h</v>
+      </c>
+      <c r="AB13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AC13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AE13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AF13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG13" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AH13" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="str">
         <f t="shared" si="1"/>
         <v>16h</v>
       </c>
-      <c r="U9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="V9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="W9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="X9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="Y9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AA9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AB9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AC9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AD9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AE9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AF9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AG9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AH9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AI9" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ9" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="AI14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AK14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AM14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AO14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AQ14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AR14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AS14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AT14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AU14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AV14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AW14" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AX14" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
         <v>22</v>
       </c>
-      <c r="B10" t="str">
+      <c r="AI15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AK15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AM15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AO15" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP15" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:50" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" t="s">
+        <v>22</v>
+      </c>
+      <c r="AI16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AJ16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AK16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AL16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AM16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AN16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AO16" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AP16" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:66" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="str">
         <f t="shared" si="1"/>
         <v>8h</v>
       </c>
-      <c r="AI10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AM10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AN10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO10" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AP10" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" t="str">
-        <f t="shared" si="1"/>
-        <v>7h</v>
-      </c>
-      <c r="AJ11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AM11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AN11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO11" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AP11" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" t="str">
-        <f t="shared" si="1"/>
-        <v>7h</v>
-      </c>
-      <c r="AJ12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AM12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AN12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO12" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AP12" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" t="str">
-        <f t="shared" si="1"/>
-        <v>16h</v>
-      </c>
-      <c r="AI13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AJ13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AK13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AL13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AM13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AN13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AO13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AP13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AQ13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AR13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AS13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AT13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AU13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AV13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AW13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AX13" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" t="str">
-        <f t="shared" si="1"/>
-        <v>6h</v>
-      </c>
-      <c r="AQ14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AR14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AS14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AT14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AU14" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AV14" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" t="str">
-        <f t="shared" si="1"/>
-        <v>6h</v>
-      </c>
-      <c r="AQ15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AR15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AS15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AT15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AU15" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AV15" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:50" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" t="str">
-        <f t="shared" si="1"/>
-        <v>2h</v>
-      </c>
-      <c r="AW16" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AX16" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:66" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" t="str">
-        <f t="shared" si="1"/>
-        <v>16h</v>
-      </c>
-      <c r="AY17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AZ17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BA17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BB17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BC17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BD17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BE17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BF17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BG17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BH17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BI17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BJ17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BK17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BL17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BM17" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BN17" s="2" t="s">
+      <c r="AQ17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AR17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AS17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AT17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AU17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AV17" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="AW17" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="AX17" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:66" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B18" t="str">
-        <f t="shared" si="1"/>
-        <v>4h</v>
-      </c>
-      <c r="AY18" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="AZ18" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BA18" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BB18" s="2" t="s">
+        <f>_xlfn.CONCAT(COUNTIF($C18:$XFD18,"x"),"h")</f>
+        <v>8h</v>
+      </c>
+      <c r="AQ18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AR18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AS18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AT18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AU18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AV18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AW18" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AX18" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:66" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B19" t="str">
-        <f t="shared" si="1"/>
-        <v>5h</v>
+        <f>_xlfn.CONCAT(COUNTIF($C19:$XFD19,"x"),"h")</f>
+        <v>16h</v>
+      </c>
+      <c r="AY19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AZ19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BA19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BB19" s="2" t="s">
+        <v>3</v>
       </c>
       <c r="BC19" s="2" t="s">
         <v>3</v>
@@ -1293,54 +1302,128 @@
         <v>3</v>
       </c>
       <c r="BG19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BH19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BI19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BJ19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BK19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BL19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BM19" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BN19" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:66" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B20" t="str">
-        <f t="shared" si="1"/>
-        <v>3h</v>
-      </c>
-      <c r="BH20" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BI20" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BJ20" s="2" t="s">
+        <f>_xlfn.CONCAT(COUNTIF($C20:$XFD20,"x"),"h")</f>
+        <v>4h</v>
+      </c>
+      <c r="AY20" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AZ20" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BA20" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BB20" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:66" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B21" t="str">
-        <f t="shared" si="1"/>
-        <v>4h</v>
-      </c>
-      <c r="BK21" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BL21" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BM21" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="BN21" s="2" t="s">
+        <f>_xlfn.CONCAT(COUNTIF($C21:$XFD21,"x"),"h")</f>
+        <v>7h</v>
+      </c>
+      <c r="BC21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BD21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BE21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BF21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BG21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BH21" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BI21" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:66" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" t="str">
+        <f>_xlfn.CONCAT(COUNTIF($C22:$XFD22,"x"),"h")</f>
+        <v>3h</v>
+      </c>
+      <c r="BJ22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BK22" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BL22" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:66" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="str">
+        <f>_xlfn.CONCAT(COUNTIF($C23:$XFD23,"x"),"h")</f>
+        <v>2h</v>
+      </c>
+      <c r="BK23" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BL23" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:66" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+      <c r="BM24" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="BN24" s="2" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A13:AV13 AW13:AX14 AY13:XFD13">
-    <cfRule type="containsText" priority="16" operator="containsText" text="x">
-      <formula>NOT(ISERROR(SEARCH("x",A13)))</formula>
-    </cfRule>
-    <cfRule type="colorScale" priority="17">
+  <conditionalFormatting sqref="A14:XFD14 AW17:AX17">
+    <cfRule type="colorScale" priority="22">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1349,8 +1432,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A17:AV17 BO17:XFD17">
-    <cfRule type="colorScale" priority="13">
+  <conditionalFormatting sqref="A14:XFD14 AW17:AX17">
+    <cfRule type="containsText" priority="21" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A14)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A19:AV19 BO19:XFD19">
+    <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1359,22 +1447,32 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:BK6 A18:BK19 BH20:BK20 A21:BK21 BM4:XFD6 BM8:XFD12 BM14:XFD16 BM18:XFD21 A8:BK12 A14:BK16">
-    <cfRule type="containsText" dxfId="11" priority="22" operator="containsText" text="x">
+  <conditionalFormatting sqref="A22:BF22 A9:XFD12 AQ13:XFD13 A13:AI13">
+    <cfRule type="containsText" dxfId="16" priority="6" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A9)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20:BK21 BH22:BK22 A23:BK23 A17:BK18 A24">
+    <cfRule type="containsText" dxfId="2" priority="27" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A17)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4:XFD6 BL17:XFD18 BL20:XFD23">
+    <cfRule type="containsText" dxfId="15" priority="7" operator="containsText" text="x">
       <formula>NOT(ISERROR(SEARCH("x",A4)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A7:XFD7">
-    <cfRule type="containsText" dxfId="10" priority="18" operator="containsText" text="x">
+  <conditionalFormatting sqref="A7:XFD7 B8:R8 U8:XFD8">
+    <cfRule type="containsText" dxfId="14" priority="23" operator="containsText" text="x">
       <formula>NOT(ISERROR(SEARCH("x",A7)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="19" operator="containsText" text="x">
+    <cfRule type="containsText" dxfId="13" priority="24" operator="containsText" text="x">
       <formula>NOT(ISERROR(SEARCH("x",A7)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="20" operator="containsText" text="x">
+    <cfRule type="containsText" priority="25" operator="containsText" text="x">
       <formula>NOT(ISERROR(SEARCH("x",A7)))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="21">
+    <cfRule type="colorScale" priority="26">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1383,33 +1481,41 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A17:XFD17">
-    <cfRule type="containsText" dxfId="8" priority="4" operator="containsText" text="x">
-      <formula>NOT(ISERROR(SEARCH("x",A17)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="x">
-      <formula>NOT(ISERROR(SEARCH("x",A17)))</formula>
-    </cfRule>
-    <cfRule type="containsText" priority="6" operator="containsText" text="x">
-      <formula>NOT(ISERROR(SEARCH("x",A17)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3:F3 A20:AR20 AT20:BF20">
-    <cfRule type="containsText" dxfId="6" priority="24" operator="containsText" text="x">
-      <formula>NOT(ISERROR(SEARCH("x",A3)))</formula>
+  <conditionalFormatting sqref="A14:XFD14 AW17:AX17">
+    <cfRule type="containsText" dxfId="12" priority="19" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A14)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="11" priority="20" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A14)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A19:XFD19">
+    <cfRule type="containsText" dxfId="10" priority="9" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="9" priority="10" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A19)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="11" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A19)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:F3">
+    <cfRule type="containsText" dxfId="8" priority="29" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",C3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:R2">
-    <cfRule type="containsText" dxfId="5" priority="29" operator="containsText" text="x">
+    <cfRule type="containsText" dxfId="7" priority="34" operator="containsText" text="x">
       <formula>NOT(ISERROR(SEARCH("x",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="30" operator="containsText" text="x">
+    <cfRule type="containsText" dxfId="6" priority="35" operator="containsText" text="x">
       <formula>NOT(ISERROR(SEARCH("x",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="31" operator="containsText" text="x">
+    <cfRule type="containsText" priority="36" operator="containsText" text="x">
       <formula>NOT(ISERROR(SEARCH("x",C2)))</formula>
     </cfRule>
-    <cfRule type="colorScale" priority="32">
+    <cfRule type="colorScale" priority="37">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1418,16 +1524,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AW14:AX14 A13:XFD13">
-    <cfRule type="containsText" dxfId="3" priority="14" operator="containsText" text="x">
-      <formula>NOT(ISERROR(SEARCH("x",A13)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="15" operator="containsText" text="x">
-      <formula>NOT(ISERROR(SEARCH("x",A13)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AW17:BN17">
-    <cfRule type="colorScale" priority="73">
+  <conditionalFormatting sqref="AW19:BN19">
+    <cfRule type="colorScale" priority="78">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -1436,14 +1534,29 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BL4:BL6 BL8:BL12 BL14:BL16 BL18:BL21">
+  <conditionalFormatting sqref="A8">
+    <cfRule type="containsText" dxfId="5" priority="5" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A8)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S8:T8">
+    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",S8)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A15:XFD16">
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="x">
+      <formula>NOT(ISERROR(SEARCH("x",A15)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BM24:BN24">
     <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="x">
-      <formula>NOT(ISERROR(SEARCH("x",BL4)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AS20">
+      <formula>NOT(ISERROR(SEARCH("x",BM24)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BK24:BL24">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="x">
-      <formula>NOT(ISERROR(SEARCH("x",AS20)))</formula>
+      <formula>NOT(ISERROR(SEARCH("x",BK24)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>